<commit_message>
add fasta for favalli
</commit_message>
<xml_diff>
--- a/supporting_material/experiments/favalli/lane-1-fasta.xlsx
+++ b/supporting_material/experiments/favalli/lane-1-fasta.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adrianomartinelli/projects/delt-hit/supporting_material/experiments/favalli/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03529B5E-D540-1E48-8187-2D5B76997732}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E7E758F-9E50-4C4A-B277-F301941CC76C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="15120" yWindow="660" windowWidth="15120" windowHeight="18980" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2968,9 +2968,6 @@
     <t>TGGCAAT</t>
   </si>
   <si>
-    <t>lane-1</t>
-  </si>
-  <si>
     <t>./</t>
   </si>
   <si>
@@ -4592,6 +4589,9 @@
   </si>
   <si>
     <t>./20190812.A-1907_NF2GB2_s1_R1.fasta.gz</t>
+  </si>
+  <si>
+    <t>lane-1-fasta</t>
   </si>
 </sst>
 </file>
@@ -5253,7 +5253,7 @@
         <v>14</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>974</v>
+        <v>1515</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -5261,7 +5261,7 @@
         <v>23</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>1515</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -5269,7 +5269,7 @@
         <v>24</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.25">
@@ -5308,15 +5308,15 @@
         <v>19</v>
       </c>
       <c r="D1" s="41" t="s">
+        <v>1512</v>
+      </c>
+      <c r="E1" s="41" t="s">
         <v>1513</v>
-      </c>
-      <c r="E1" s="41" t="s">
-        <v>1514</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="18" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="B2" s="18" t="s">
         <v>34</v>
@@ -5327,7 +5327,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="18" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
       <c r="B3" s="18" t="s">
         <v>35</v>
@@ -5338,7 +5338,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="18" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="B4" s="18" t="s">
         <v>36</v>
@@ -5349,7 +5349,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="18" t="s">
-        <v>982</v>
+        <v>981</v>
       </c>
       <c r="B5" s="18" t="s">
         <v>6</v>
@@ -5360,7 +5360,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="18" t="s">
-        <v>983</v>
+        <v>982</v>
       </c>
       <c r="B6" s="18" t="s">
         <v>8</v>
@@ -5371,7 +5371,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="18" t="s">
-        <v>984</v>
+        <v>983</v>
       </c>
       <c r="B7" s="18" t="s">
         <v>37</v>
@@ -5382,7 +5382,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="18" t="s">
-        <v>985</v>
+        <v>984</v>
       </c>
       <c r="B8" s="18" t="s">
         <v>3</v>
@@ -5393,7 +5393,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="18" t="s">
-        <v>986</v>
+        <v>985</v>
       </c>
       <c r="B9" s="18" t="s">
         <v>38</v>
@@ -5404,7 +5404,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="18" t="s">
-        <v>987</v>
+        <v>986</v>
       </c>
       <c r="B10" s="18" t="s">
         <v>39</v>
@@ -5415,7 +5415,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="18" t="s">
-        <v>988</v>
+        <v>987</v>
       </c>
       <c r="B11" s="18" t="s">
         <v>40</v>
@@ -5426,7 +5426,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="18" t="s">
-        <v>989</v>
+        <v>988</v>
       </c>
       <c r="B12" s="18" t="s">
         <v>41</v>
@@ -5437,7 +5437,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="18" t="s">
-        <v>990</v>
+        <v>989</v>
       </c>
       <c r="B13" s="18" t="s">
         <v>42</v>
@@ -5448,7 +5448,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" s="18" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
       <c r="B14" s="18" t="s">
         <v>43</v>
@@ -5459,7 +5459,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" s="18" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
       <c r="B15" s="18" t="s">
         <v>44</v>
@@ -5470,7 +5470,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" s="18" t="s">
-        <v>993</v>
+        <v>992</v>
       </c>
       <c r="B16" s="18" t="s">
         <v>45</v>
@@ -5481,7 +5481,7 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="18" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="B17" s="18" t="s">
         <v>46</v>
@@ -5492,7 +5492,7 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="18" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="B18" s="18" t="s">
         <v>47</v>
@@ -5503,7 +5503,7 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="18" t="s">
-        <v>996</v>
+        <v>995</v>
       </c>
       <c r="B19" s="18" t="s">
         <v>48</v>
@@ -5514,7 +5514,7 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="18" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
       <c r="B20" s="18" t="s">
         <v>49</v>
@@ -5525,7 +5525,7 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="18" t="s">
-        <v>998</v>
+        <v>997</v>
       </c>
       <c r="B21" s="18" t="s">
         <v>50</v>
@@ -5536,7 +5536,7 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="18" t="s">
-        <v>999</v>
+        <v>998</v>
       </c>
       <c r="B22" s="18" t="s">
         <v>51</v>
@@ -5547,7 +5547,7 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="18" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="B23" s="18" t="s">
         <v>52</v>
@@ -5558,7 +5558,7 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="18" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
       <c r="B24" s="18" t="s">
         <v>9</v>
@@ -5569,7 +5569,7 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" s="18" t="s">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="B25" s="18" t="s">
         <v>7</v>
@@ -5580,7 +5580,7 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" s="18" t="s">
-        <v>1003</v>
+        <v>1002</v>
       </c>
       <c r="B26" s="18" t="s">
         <v>53</v>
@@ -5591,7 +5591,7 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" s="18" t="s">
-        <v>1004</v>
+        <v>1003</v>
       </c>
       <c r="B27" s="18" t="s">
         <v>54</v>
@@ -5602,7 +5602,7 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" s="18" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="B28" s="18" t="s">
         <v>55</v>
@@ -5613,7 +5613,7 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" s="18" t="s">
-        <v>1006</v>
+        <v>1005</v>
       </c>
       <c r="B29" s="18" t="s">
         <v>61</v>
@@ -5624,7 +5624,7 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" s="18" t="s">
-        <v>1007</v>
+        <v>1006</v>
       </c>
       <c r="B30" s="18" t="s">
         <v>58</v>
@@ -5635,7 +5635,7 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" s="18" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
       <c r="B31" s="18" t="s">
         <v>59</v>
@@ -5646,7 +5646,7 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" s="18" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
       <c r="B32" s="18" t="s">
         <v>62</v>
@@ -5657,7 +5657,7 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" s="18" t="s">
-        <v>1010</v>
+        <v>1009</v>
       </c>
       <c r="B33" s="18" t="s">
         <v>64</v>
@@ -5668,7 +5668,7 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" s="18" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
       <c r="B34" s="18" t="s">
         <v>65</v>
@@ -5679,7 +5679,7 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" s="18" t="s">
-        <v>1012</v>
+        <v>1011</v>
       </c>
       <c r="B35" s="18" t="s">
         <v>71</v>
@@ -5690,7 +5690,7 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A36" s="18" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
       <c r="B36" s="18" t="s">
         <v>72</v>
@@ -5701,7 +5701,7 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" s="18" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
       <c r="B37" s="18" t="s">
         <v>79</v>
@@ -5712,7 +5712,7 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A38" s="18" t="s">
-        <v>1015</v>
+        <v>1014</v>
       </c>
       <c r="B38" s="18" t="s">
         <v>96</v>
@@ -5723,7 +5723,7 @@
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A39" s="18" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
       <c r="B39" s="18" t="s">
         <v>121</v>
@@ -5734,7 +5734,7 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A40" s="18" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
       <c r="B40" s="18" t="s">
         <v>75</v>
@@ -5745,7 +5745,7 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A41" s="18" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
       <c r="B41" s="18" t="s">
         <v>69</v>
@@ -5756,7 +5756,7 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A42" s="18" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
       <c r="B42" s="18" t="s">
         <v>115</v>
@@ -5767,7 +5767,7 @@
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A43" s="18" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
       <c r="B43" s="18" t="s">
         <v>76</v>
@@ -5778,7 +5778,7 @@
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A44" s="18" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
       <c r="B44" s="18" t="s">
         <v>106</v>
@@ -5789,7 +5789,7 @@
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A45" s="18" t="s">
-        <v>1022</v>
+        <v>1021</v>
       </c>
       <c r="B45" s="18" t="s">
         <v>88</v>
@@ -5800,7 +5800,7 @@
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A46" s="18" t="s">
-        <v>1023</v>
+        <v>1022</v>
       </c>
       <c r="B46" s="18" t="s">
         <v>116</v>
@@ -5811,7 +5811,7 @@
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A47" s="18" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
       <c r="B47" s="18" t="s">
         <v>109</v>
@@ -5822,7 +5822,7 @@
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A48" s="18" t="s">
-        <v>1025</v>
+        <v>1024</v>
       </c>
       <c r="B48" s="18" t="s">
         <v>113</v>
@@ -5833,7 +5833,7 @@
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A49" s="18" t="s">
-        <v>1026</v>
+        <v>1025</v>
       </c>
       <c r="B49" s="18" t="s">
         <v>126</v>
@@ -5844,7 +5844,7 @@
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A50" s="18" t="s">
-        <v>1027</v>
+        <v>1026</v>
       </c>
       <c r="B50" s="18" t="s">
         <v>118</v>
@@ -5855,7 +5855,7 @@
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A51" s="18" t="s">
-        <v>1028</v>
+        <v>1027</v>
       </c>
       <c r="B51" s="18" t="s">
         <v>83</v>
@@ -5866,7 +5866,7 @@
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A52" s="18" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="B52" s="18" t="s">
         <v>92</v>
@@ -5877,7 +5877,7 @@
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A53" s="18" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="B53" s="18" t="s">
         <v>102</v>
@@ -5888,7 +5888,7 @@
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A54" s="18" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="B54" s="18" t="s">
         <v>67</v>
@@ -5899,7 +5899,7 @@
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A55" s="18" t="s">
-        <v>1032</v>
+        <v>1031</v>
       </c>
       <c r="B55" s="18" t="s">
         <v>110</v>
@@ -5910,7 +5910,7 @@
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A56" s="18" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
       <c r="B56" s="18" t="s">
         <v>122</v>
@@ -5921,7 +5921,7 @@
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A57" s="18" t="s">
-        <v>1034</v>
+        <v>1033</v>
       </c>
       <c r="B57" s="18" t="s">
         <v>105</v>
@@ -5932,7 +5932,7 @@
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A58" s="18" t="s">
-        <v>1035</v>
+        <v>1034</v>
       </c>
       <c r="B58" s="18" t="s">
         <v>123</v>
@@ -5943,7 +5943,7 @@
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A59" s="18" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
       <c r="B59" s="18" t="s">
         <v>127</v>
@@ -5954,7 +5954,7 @@
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A60" s="18" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
       <c r="B60" s="18" t="s">
         <v>125</v>
@@ -5965,7 +5965,7 @@
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A61" s="18" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="B61" s="18" t="s">
         <v>128</v>
@@ -5976,7 +5976,7 @@
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A62" s="18" t="s">
-        <v>1039</v>
+        <v>1038</v>
       </c>
       <c r="B62" s="18" t="s">
         <v>87</v>
@@ -5987,7 +5987,7 @@
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A63" s="18" t="s">
-        <v>1040</v>
+        <v>1039</v>
       </c>
       <c r="B63" s="18" t="s">
         <v>111</v>
@@ -5998,7 +5998,7 @@
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A64" s="18" t="s">
-        <v>1041</v>
+        <v>1040</v>
       </c>
       <c r="B64" s="18" t="s">
         <v>124</v>
@@ -6009,7 +6009,7 @@
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A65" s="18" t="s">
-        <v>1042</v>
+        <v>1041</v>
       </c>
       <c r="B65" s="18" t="s">
         <v>82</v>
@@ -6020,7 +6020,7 @@
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A66" s="18" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
       <c r="B66" s="18" t="s">
         <v>97</v>
@@ -6031,7 +6031,7 @@
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A67" s="18" t="s">
-        <v>1044</v>
+        <v>1043</v>
       </c>
       <c r="B67" s="18" t="s">
         <v>68</v>
@@ -6042,7 +6042,7 @@
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A68" s="18" t="s">
-        <v>1045</v>
+        <v>1044</v>
       </c>
       <c r="B68" s="18" t="s">
         <v>98</v>
@@ -6053,7 +6053,7 @@
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A69" s="18" t="s">
-        <v>1046</v>
+        <v>1045</v>
       </c>
       <c r="B69" s="18" t="s">
         <v>77</v>
@@ -6064,7 +6064,7 @@
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A70" s="18" t="s">
-        <v>1047</v>
+        <v>1046</v>
       </c>
       <c r="B70" s="18" t="s">
         <v>89</v>
@@ -6075,7 +6075,7 @@
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A71" s="18" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="B71" s="18" t="s">
         <v>107</v>
@@ -6086,7 +6086,7 @@
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A72" s="18" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
       <c r="B72" s="18" t="s">
         <v>84</v>
@@ -6097,7 +6097,7 @@
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A73" s="18" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
       <c r="B73" s="18" t="s">
         <v>103</v>
@@ -6108,7 +6108,7 @@
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A74" s="18" t="s">
-        <v>1051</v>
+        <v>1050</v>
       </c>
       <c r="B74" s="18" t="s">
         <v>114</v>
@@ -6119,7 +6119,7 @@
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A75" s="18" t="s">
-        <v>1052</v>
+        <v>1051</v>
       </c>
       <c r="B75" s="18" t="s">
         <v>66</v>
@@ -6130,7 +6130,7 @@
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A76" s="18" t="s">
-        <v>1053</v>
+        <v>1052</v>
       </c>
       <c r="B76" s="18" t="s">
         <v>85</v>
@@ -6141,7 +6141,7 @@
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A77" s="18" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
       <c r="B77" s="18" t="s">
         <v>108</v>
@@ -6152,7 +6152,7 @@
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A78" s="18" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="B78" s="18" t="s">
         <v>101</v>
@@ -6163,7 +6163,7 @@
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A79" s="18" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
       <c r="B79" s="18" t="s">
         <v>73</v>
@@ -6174,7 +6174,7 @@
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A80" s="18" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="B80" s="18" t="s">
         <v>99</v>
@@ -6185,7 +6185,7 @@
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A81" s="18" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="B81" s="18" t="s">
         <v>74</v>
@@ -6196,7 +6196,7 @@
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A82" s="18" t="s">
-        <v>1059</v>
+        <v>1058</v>
       </c>
       <c r="B82" s="18" t="s">
         <v>86</v>
@@ -6207,7 +6207,7 @@
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A83" s="18" t="s">
-        <v>1060</v>
+        <v>1059</v>
       </c>
       <c r="B83" s="18" t="s">
         <v>100</v>
@@ -6218,7 +6218,7 @@
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A84" s="18" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
       <c r="B84" s="18" t="s">
         <v>70</v>
@@ -6229,7 +6229,7 @@
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A85" s="18" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="B85" s="18" t="s">
         <v>78</v>
@@ -6240,7 +6240,7 @@
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A86" s="18" t="s">
-        <v>1063</v>
+        <v>1062</v>
       </c>
       <c r="B86" s="18" t="s">
         <v>90</v>
@@ -6251,7 +6251,7 @@
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A87" s="18" t="s">
-        <v>1064</v>
+        <v>1063</v>
       </c>
       <c r="B87" s="18" t="s">
         <v>104</v>
@@ -6262,7 +6262,7 @@
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A88" s="18" t="s">
-        <v>1065</v>
+        <v>1064</v>
       </c>
       <c r="B88" s="18" t="s">
         <v>112</v>
@@ -6273,7 +6273,7 @@
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A89" s="18" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="B89" s="18" t="s">
         <v>80</v>
@@ -6284,7 +6284,7 @@
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A90" s="18" t="s">
-        <v>1067</v>
+        <v>1066</v>
       </c>
       <c r="B90" s="18" t="s">
         <v>95</v>
@@ -6295,7 +6295,7 @@
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A91" s="18" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="B91" s="18" t="s">
         <v>81</v>
@@ -6306,7 +6306,7 @@
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A92" s="18" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="B92" s="18" t="s">
         <v>117</v>
@@ -6317,7 +6317,7 @@
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A93" s="18" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="B93" s="18" t="s">
         <v>91</v>
@@ -6328,7 +6328,7 @@
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A94" s="18" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
       <c r="B94" s="18" t="s">
         <v>120</v>
@@ -6339,7 +6339,7 @@
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A95" s="18" t="s">
-        <v>1072</v>
+        <v>1071</v>
       </c>
       <c r="B95" s="18" t="s">
         <v>119</v>
@@ -6350,7 +6350,7 @@
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A96" s="18" t="s">
-        <v>1073</v>
+        <v>1072</v>
       </c>
       <c r="B96" s="18" t="s">
         <v>93</v>
@@ -6361,7 +6361,7 @@
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A97" s="18" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
       <c r="B97" s="18" t="s">
         <v>94</v>
@@ -6372,7 +6372,7 @@
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A98" s="18" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="B98" s="18" t="s">
         <v>34</v>
@@ -6381,12 +6381,12 @@
         <v>422</v>
       </c>
       <c r="D98" s="42" t="s">
-        <v>1468</v>
+        <v>1467</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A99" s="18" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
       <c r="B99" s="18" t="s">
         <v>35</v>
@@ -6395,12 +6395,12 @@
         <v>422</v>
       </c>
       <c r="D99" s="42" t="s">
-        <v>1468</v>
+        <v>1467</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A100" s="18" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="B100" s="18" t="s">
         <v>36</v>
@@ -6409,12 +6409,12 @@
         <v>422</v>
       </c>
       <c r="D100" s="42" t="s">
-        <v>1468</v>
+        <v>1467</v>
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A101" s="18" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
       <c r="B101" s="18" t="s">
         <v>6</v>
@@ -6423,15 +6423,15 @@
         <v>422</v>
       </c>
       <c r="D101" s="42" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="E101" s="39" t="s">
-        <v>1469</v>
+        <v>1468</v>
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A102" s="18" t="s">
-        <v>1076</v>
+        <v>1075</v>
       </c>
       <c r="B102" s="18" t="s">
         <v>8</v>
@@ -6440,15 +6440,15 @@
         <v>422</v>
       </c>
       <c r="D102" s="42" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="E102" s="39" t="s">
-        <v>1469</v>
+        <v>1468</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A103" s="18" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
       <c r="B103" s="18" t="s">
         <v>37</v>
@@ -6457,15 +6457,15 @@
         <v>422</v>
       </c>
       <c r="D103" s="42" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
       <c r="E103" s="39" t="s">
-        <v>1469</v>
+        <v>1468</v>
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A104" s="18" t="s">
-        <v>1078</v>
+        <v>1077</v>
       </c>
       <c r="B104" s="18" t="s">
         <v>3</v>
@@ -6474,12 +6474,12 @@
         <v>422</v>
       </c>
       <c r="D104" s="42" t="s">
-        <v>1471</v>
+        <v>1470</v>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A105" s="18" t="s">
-        <v>1079</v>
+        <v>1078</v>
       </c>
       <c r="B105" s="18" t="s">
         <v>38</v>
@@ -6488,12 +6488,12 @@
         <v>422</v>
       </c>
       <c r="D105" s="42" t="s">
-        <v>1472</v>
+        <v>1471</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A106" s="18" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
       <c r="B106" s="18" t="s">
         <v>39</v>
@@ -6502,12 +6502,12 @@
         <v>422</v>
       </c>
       <c r="D106" s="42" t="s">
-        <v>1473</v>
+        <v>1472</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A107" s="18" t="s">
-        <v>1081</v>
+        <v>1080</v>
       </c>
       <c r="B107" s="18" t="s">
         <v>40</v>
@@ -6516,12 +6516,12 @@
         <v>422</v>
       </c>
       <c r="D107" s="42" t="s">
-        <v>1474</v>
+        <v>1473</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A108" s="18" t="s">
-        <v>1082</v>
+        <v>1081</v>
       </c>
       <c r="B108" s="18" t="s">
         <v>41</v>
@@ -6530,12 +6530,12 @@
         <v>422</v>
       </c>
       <c r="D108" s="42" t="s">
-        <v>1474</v>
+        <v>1473</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A109" s="18" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="B109" s="18" t="s">
         <v>42</v>
@@ -6544,12 +6544,12 @@
         <v>422</v>
       </c>
       <c r="D109" s="42" t="s">
-        <v>1474</v>
+        <v>1473</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A110" s="18" t="s">
-        <v>1084</v>
+        <v>1083</v>
       </c>
       <c r="B110" s="18" t="s">
         <v>43</v>
@@ -6558,12 +6558,12 @@
         <v>422</v>
       </c>
       <c r="D110" s="42" t="s">
-        <v>1476</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A111" s="18" t="s">
-        <v>1085</v>
+        <v>1084</v>
       </c>
       <c r="B111" s="18" t="s">
         <v>44</v>
@@ -6572,12 +6572,12 @@
         <v>422</v>
       </c>
       <c r="D111" s="42" t="s">
-        <v>1476</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A112" s="18" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="B112" s="18" t="s">
         <v>45</v>
@@ -6586,12 +6586,12 @@
         <v>422</v>
       </c>
       <c r="D112" s="42" t="s">
-        <v>1476</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A113" s="18" t="s">
-        <v>1087</v>
+        <v>1086</v>
       </c>
       <c r="B113" s="18" t="s">
         <v>46</v>
@@ -6600,12 +6600,12 @@
         <v>422</v>
       </c>
       <c r="D113" s="42" t="s">
-        <v>1477</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A114" s="18" t="s">
-        <v>1088</v>
+        <v>1087</v>
       </c>
       <c r="B114" s="18" t="s">
         <v>47</v>
@@ -6614,12 +6614,12 @@
         <v>422</v>
       </c>
       <c r="D114" s="42" t="s">
-        <v>1477</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A115" s="18" t="s">
-        <v>1089</v>
+        <v>1088</v>
       </c>
       <c r="B115" s="18" t="s">
         <v>48</v>
@@ -6628,12 +6628,12 @@
         <v>422</v>
       </c>
       <c r="D115" s="42" t="s">
-        <v>1477</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A116" s="18" t="s">
-        <v>1090</v>
+        <v>1089</v>
       </c>
       <c r="B116" s="18" t="s">
         <v>49</v>
@@ -6642,12 +6642,12 @@
         <v>422</v>
       </c>
       <c r="D116" s="42" t="s">
-        <v>1478</v>
+        <v>1477</v>
       </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A117" s="18" t="s">
-        <v>1091</v>
+        <v>1090</v>
       </c>
       <c r="B117" s="18" t="s">
         <v>50</v>
@@ -6656,12 +6656,12 @@
         <v>422</v>
       </c>
       <c r="D117" s="42" t="s">
-        <v>1479</v>
+        <v>1478</v>
       </c>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A118" s="18" t="s">
-        <v>1092</v>
+        <v>1091</v>
       </c>
       <c r="B118" s="18" t="s">
         <v>51</v>
@@ -6670,12 +6670,12 @@
         <v>422</v>
       </c>
       <c r="D118" s="42" t="s">
-        <v>1480</v>
+        <v>1479</v>
       </c>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A119" s="18" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
       <c r="B119" s="18" t="s">
         <v>52</v>
@@ -6684,15 +6684,15 @@
         <v>422</v>
       </c>
       <c r="D119" s="42" t="s">
-        <v>1481</v>
+        <v>1480</v>
       </c>
       <c r="E119" s="40" t="s">
-        <v>1475</v>
+        <v>1474</v>
       </c>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A120" s="18" t="s">
-        <v>1094</v>
+        <v>1093</v>
       </c>
       <c r="B120" s="18" t="s">
         <v>9</v>
@@ -6701,15 +6701,15 @@
         <v>422</v>
       </c>
       <c r="D120" s="42" t="s">
-        <v>1481</v>
+        <v>1480</v>
       </c>
       <c r="E120" s="40" t="s">
-        <v>1475</v>
+        <v>1474</v>
       </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A121" s="18" t="s">
-        <v>1095</v>
+        <v>1094</v>
       </c>
       <c r="B121" s="18" t="s">
         <v>7</v>
@@ -6718,15 +6718,15 @@
         <v>422</v>
       </c>
       <c r="D121" s="42" t="s">
-        <v>1481</v>
+        <v>1480</v>
       </c>
       <c r="E121" s="40" t="s">
-        <v>1475</v>
+        <v>1474</v>
       </c>
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A122" s="18" t="s">
-        <v>1096</v>
+        <v>1095</v>
       </c>
       <c r="B122" s="18" t="s">
         <v>53</v>
@@ -6735,12 +6735,12 @@
         <v>422</v>
       </c>
       <c r="D122" s="42" t="s">
-        <v>1482</v>
+        <v>1481</v>
       </c>
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A123" s="18" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="B123" s="18" t="s">
         <v>54</v>
@@ -6749,12 +6749,12 @@
         <v>422</v>
       </c>
       <c r="D123" s="42" t="s">
-        <v>1482</v>
+        <v>1481</v>
       </c>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A124" s="18" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
       <c r="B124" s="18" t="s">
         <v>55</v>
@@ -6763,12 +6763,12 @@
         <v>422</v>
       </c>
       <c r="D124" s="42" t="s">
-        <v>1482</v>
+        <v>1481</v>
       </c>
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A125" s="18" t="s">
-        <v>1099</v>
+        <v>1098</v>
       </c>
       <c r="B125" s="18" t="s">
         <v>61</v>
@@ -6777,12 +6777,12 @@
         <v>422</v>
       </c>
       <c r="D125" s="42" t="s">
-        <v>1483</v>
+        <v>1482</v>
       </c>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A126" s="18" t="s">
-        <v>1100</v>
+        <v>1099</v>
       </c>
       <c r="B126" s="18" t="s">
         <v>58</v>
@@ -6791,12 +6791,12 @@
         <v>422</v>
       </c>
       <c r="D126" s="42" t="s">
-        <v>1483</v>
+        <v>1482</v>
       </c>
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A127" s="18" t="s">
-        <v>1101</v>
+        <v>1100</v>
       </c>
       <c r="B127" s="18" t="s">
         <v>59</v>
@@ -6805,12 +6805,12 @@
         <v>422</v>
       </c>
       <c r="D127" s="42" t="s">
-        <v>1483</v>
+        <v>1482</v>
       </c>
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A128" s="18" t="s">
-        <v>1102</v>
+        <v>1101</v>
       </c>
       <c r="B128" s="18" t="s">
         <v>62</v>
@@ -6819,12 +6819,12 @@
         <v>422</v>
       </c>
       <c r="D128" s="42" t="s">
-        <v>1484</v>
+        <v>1483</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A129" s="18" t="s">
-        <v>1103</v>
+        <v>1102</v>
       </c>
       <c r="B129" s="18" t="s">
         <v>64</v>
@@ -6833,12 +6833,12 @@
         <v>422</v>
       </c>
       <c r="D129" s="42" t="s">
-        <v>1484</v>
+        <v>1483</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A130" s="18" t="s">
-        <v>1104</v>
+        <v>1103</v>
       </c>
       <c r="B130" s="18" t="s">
         <v>65</v>
@@ -6847,12 +6847,12 @@
         <v>422</v>
       </c>
       <c r="D130" s="42" t="s">
-        <v>1484</v>
+        <v>1483</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A131" s="18" t="s">
-        <v>1105</v>
+        <v>1104</v>
       </c>
       <c r="B131" s="18" t="s">
         <v>71</v>
@@ -6861,12 +6861,12 @@
         <v>422</v>
       </c>
       <c r="D131" s="42" t="s">
-        <v>1485</v>
+        <v>1484</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A132" s="18" t="s">
-        <v>1106</v>
+        <v>1105</v>
       </c>
       <c r="B132" s="18" t="s">
         <v>72</v>
@@ -6875,12 +6875,12 @@
         <v>422</v>
       </c>
       <c r="D132" s="42" t="s">
-        <v>1486</v>
+        <v>1485</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A133" s="18" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="B133" s="18" t="s">
         <v>79</v>
@@ -6889,12 +6889,12 @@
         <v>422</v>
       </c>
       <c r="D133" s="42" t="s">
-        <v>1487</v>
+        <v>1486</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A134" s="18" t="s">
-        <v>1108</v>
+        <v>1107</v>
       </c>
       <c r="B134" s="18" t="s">
         <v>96</v>
@@ -6903,12 +6903,12 @@
         <v>422</v>
       </c>
       <c r="D134" s="42" t="s">
-        <v>1488</v>
+        <v>1487</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A135" s="18" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="B135" s="18" t="s">
         <v>121</v>
@@ -6917,12 +6917,12 @@
         <v>422</v>
       </c>
       <c r="D135" s="42" t="s">
-        <v>1488</v>
+        <v>1487</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A136" s="18" t="s">
-        <v>1110</v>
+        <v>1109</v>
       </c>
       <c r="B136" s="18" t="s">
         <v>75</v>
@@ -6931,12 +6931,12 @@
         <v>422</v>
       </c>
       <c r="D136" s="42" t="s">
-        <v>1488</v>
+        <v>1487</v>
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A137" s="18" t="s">
-        <v>1111</v>
+        <v>1110</v>
       </c>
       <c r="B137" s="18" t="s">
         <v>69</v>
@@ -6945,12 +6945,12 @@
         <v>422</v>
       </c>
       <c r="D137" s="42" t="s">
-        <v>1489</v>
+        <v>1488</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A138" s="18" t="s">
-        <v>1112</v>
+        <v>1111</v>
       </c>
       <c r="B138" s="18" t="s">
         <v>115</v>
@@ -6959,12 +6959,12 @@
         <v>422</v>
       </c>
       <c r="D138" s="42" t="s">
-        <v>1489</v>
+        <v>1488</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A139" s="18" t="s">
-        <v>1113</v>
+        <v>1112</v>
       </c>
       <c r="B139" s="18" t="s">
         <v>76</v>
@@ -6973,12 +6973,12 @@
         <v>422</v>
       </c>
       <c r="D139" s="42" t="s">
-        <v>1489</v>
+        <v>1488</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A140" s="18" t="s">
-        <v>1114</v>
+        <v>1113</v>
       </c>
       <c r="B140" s="18" t="s">
         <v>106</v>
@@ -6987,12 +6987,12 @@
         <v>422</v>
       </c>
       <c r="D140" s="42" t="s">
-        <v>1490</v>
+        <v>1489</v>
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A141" s="18" t="s">
-        <v>1115</v>
+        <v>1114</v>
       </c>
       <c r="B141" s="18" t="s">
         <v>88</v>
@@ -7001,12 +7001,12 @@
         <v>422</v>
       </c>
       <c r="D141" s="42" t="s">
-        <v>1490</v>
+        <v>1489</v>
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A142" s="18" t="s">
-        <v>1116</v>
+        <v>1115</v>
       </c>
       <c r="B142" s="18" t="s">
         <v>116</v>
@@ -7015,12 +7015,12 @@
         <v>422</v>
       </c>
       <c r="D142" s="42" t="s">
-        <v>1490</v>
+        <v>1489</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A143" s="18" t="s">
-        <v>1117</v>
+        <v>1116</v>
       </c>
       <c r="B143" s="18" t="s">
         <v>109</v>
@@ -7029,12 +7029,12 @@
         <v>422</v>
       </c>
       <c r="D143" s="42" t="s">
-        <v>1491</v>
+        <v>1490</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A144" s="18" t="s">
-        <v>1118</v>
+        <v>1117</v>
       </c>
       <c r="B144" s="18" t="s">
         <v>113</v>
@@ -7043,12 +7043,12 @@
         <v>422</v>
       </c>
       <c r="D144" s="42" t="s">
-        <v>1491</v>
+        <v>1490</v>
       </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A145" s="18" t="s">
-        <v>1119</v>
+        <v>1118</v>
       </c>
       <c r="B145" s="18" t="s">
         <v>126</v>
@@ -7057,12 +7057,12 @@
         <v>422</v>
       </c>
       <c r="D145" s="42" t="s">
-        <v>1491</v>
+        <v>1490</v>
       </c>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A146" s="18" t="s">
-        <v>1120</v>
+        <v>1119</v>
       </c>
       <c r="B146" s="18" t="s">
         <v>118</v>
@@ -7071,12 +7071,12 @@
         <v>422</v>
       </c>
       <c r="D146" s="42" t="s">
-        <v>1492</v>
+        <v>1491</v>
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A147" s="18" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
       <c r="B147" s="18" t="s">
         <v>83</v>
@@ -7085,12 +7085,12 @@
         <v>422</v>
       </c>
       <c r="D147" s="42" t="s">
-        <v>1492</v>
+        <v>1491</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A148" s="18" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
       <c r="B148" s="18" t="s">
         <v>92</v>
@@ -7099,12 +7099,12 @@
         <v>422</v>
       </c>
       <c r="D148" s="42" t="s">
-        <v>1493</v>
+        <v>1492</v>
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A149" s="18" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
       <c r="B149" s="18" t="s">
         <v>102</v>
@@ -7113,12 +7113,12 @@
         <v>422</v>
       </c>
       <c r="D149" s="42" t="s">
-        <v>1493</v>
+        <v>1492</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A150" s="18" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
       <c r="B150" s="18" t="s">
         <v>67</v>
@@ -7127,12 +7127,12 @@
         <v>422</v>
       </c>
       <c r="D150" s="42" t="s">
-        <v>1494</v>
+        <v>1493</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A151" s="18" t="s">
-        <v>1125</v>
+        <v>1124</v>
       </c>
       <c r="B151" s="18" t="s">
         <v>110</v>
@@ -7141,12 +7141,12 @@
         <v>422</v>
       </c>
       <c r="D151" s="42" t="s">
-        <v>1494</v>
+        <v>1493</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A152" s="18" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
       <c r="B152" s="18" t="s">
         <v>122</v>
@@ -7155,12 +7155,12 @@
         <v>422</v>
       </c>
       <c r="D152" s="42" t="s">
-        <v>1495</v>
+        <v>1494</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A153" s="18" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
       <c r="B153" s="18" t="s">
         <v>105</v>
@@ -7169,12 +7169,12 @@
         <v>422</v>
       </c>
       <c r="D153" s="42" t="s">
-        <v>1495</v>
+        <v>1494</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A154" s="18" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
       <c r="B154" s="18" t="s">
         <v>123</v>
@@ -7183,12 +7183,12 @@
         <v>422</v>
       </c>
       <c r="D154" s="42" t="s">
-        <v>1496</v>
+        <v>1495</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A155" s="18" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
       <c r="B155" s="18" t="s">
         <v>127</v>
@@ -7197,12 +7197,12 @@
         <v>422</v>
       </c>
       <c r="D155" s="42" t="s">
-        <v>1496</v>
+        <v>1495</v>
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A156" s="18" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
       <c r="B156" s="18" t="s">
         <v>125</v>
@@ -7211,12 +7211,12 @@
         <v>422</v>
       </c>
       <c r="D156" s="42" t="s">
-        <v>1497</v>
+        <v>1496</v>
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A157" s="18" t="s">
-        <v>1131</v>
+        <v>1130</v>
       </c>
       <c r="B157" s="18" t="s">
         <v>128</v>
@@ -7225,12 +7225,12 @@
         <v>422</v>
       </c>
       <c r="D157" s="42" t="s">
-        <v>1497</v>
+        <v>1496</v>
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A158" s="18" t="s">
-        <v>1132</v>
+        <v>1131</v>
       </c>
       <c r="B158" s="18" t="s">
         <v>87</v>
@@ -7239,12 +7239,12 @@
         <v>422</v>
       </c>
       <c r="D158" s="42" t="s">
-        <v>1498</v>
+        <v>1497</v>
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A159" s="18" t="s">
-        <v>1133</v>
+        <v>1132</v>
       </c>
       <c r="B159" s="18" t="s">
         <v>111</v>
@@ -7253,12 +7253,12 @@
         <v>422</v>
       </c>
       <c r="D159" s="42" t="s">
-        <v>1498</v>
+        <v>1497</v>
       </c>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A160" s="18" t="s">
-        <v>1134</v>
+        <v>1133</v>
       </c>
       <c r="B160" s="18" t="s">
         <v>124</v>
@@ -7267,12 +7267,12 @@
         <v>422</v>
       </c>
       <c r="D160" s="42" t="s">
-        <v>1498</v>
+        <v>1497</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A161" s="18" t="s">
-        <v>1135</v>
+        <v>1134</v>
       </c>
       <c r="B161" s="18" t="s">
         <v>82</v>
@@ -7281,12 +7281,12 @@
         <v>422</v>
       </c>
       <c r="D161" s="42" t="s">
-        <v>1499</v>
+        <v>1498</v>
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A162" s="18" t="s">
-        <v>1136</v>
+        <v>1135</v>
       </c>
       <c r="B162" s="18" t="s">
         <v>97</v>
@@ -7295,12 +7295,12 @@
         <v>422</v>
       </c>
       <c r="D162" s="42" t="s">
-        <v>1499</v>
+        <v>1498</v>
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A163" s="18" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="B163" s="18" t="s">
         <v>68</v>
@@ -7309,12 +7309,12 @@
         <v>422</v>
       </c>
       <c r="D163" s="42" t="s">
-        <v>1500</v>
+        <v>1499</v>
       </c>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A164" s="18" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="B164" s="18" t="s">
         <v>98</v>
@@ -7323,12 +7323,12 @@
         <v>422</v>
       </c>
       <c r="D164" s="42" t="s">
-        <v>1500</v>
+        <v>1499</v>
       </c>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A165" s="18" t="s">
-        <v>1139</v>
+        <v>1138</v>
       </c>
       <c r="B165" s="18" t="s">
         <v>77</v>
@@ -7337,12 +7337,12 @@
         <v>422</v>
       </c>
       <c r="D165" s="42" t="s">
-        <v>1500</v>
+        <v>1499</v>
       </c>
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A166" s="18" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="B166" s="18" t="s">
         <v>89</v>
@@ -7351,12 +7351,12 @@
         <v>422</v>
       </c>
       <c r="D166" s="42" t="s">
-        <v>1501</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A167" s="18" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="B167" s="18" t="s">
         <v>107</v>
@@ -7365,12 +7365,12 @@
         <v>422</v>
       </c>
       <c r="D167" s="42" t="s">
-        <v>1501</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A168" s="18" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="B168" s="18" t="s">
         <v>84</v>
@@ -7379,12 +7379,12 @@
         <v>422</v>
       </c>
       <c r="D168" s="42" t="s">
-        <v>1502</v>
+        <v>1501</v>
       </c>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A169" s="18" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
       <c r="B169" s="18" t="s">
         <v>103</v>
@@ -7393,12 +7393,12 @@
         <v>422</v>
       </c>
       <c r="D169" s="42" t="s">
-        <v>1502</v>
+        <v>1501</v>
       </c>
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A170" s="18" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="B170" s="18" t="s">
         <v>114</v>
@@ -7407,12 +7407,12 @@
         <v>422</v>
       </c>
       <c r="D170" s="42" t="s">
-        <v>1503</v>
+        <v>1502</v>
       </c>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A171" s="18" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="B171" s="18" t="s">
         <v>66</v>
@@ -7421,12 +7421,12 @@
         <v>422</v>
       </c>
       <c r="D171" s="42" t="s">
-        <v>1503</v>
+        <v>1502</v>
       </c>
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A172" s="18" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
       <c r="B172" s="18" t="s">
         <v>85</v>
@@ -7435,12 +7435,12 @@
         <v>422</v>
       </c>
       <c r="D172" s="42" t="s">
-        <v>1503</v>
+        <v>1502</v>
       </c>
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A173" s="18" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
       <c r="B173" s="18" t="s">
         <v>108</v>
@@ -7449,12 +7449,12 @@
         <v>422</v>
       </c>
       <c r="D173" s="42" t="s">
-        <v>1504</v>
+        <v>1503</v>
       </c>
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A174" s="18" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="B174" s="18" t="s">
         <v>101</v>
@@ -7463,12 +7463,12 @@
         <v>422</v>
       </c>
       <c r="D174" s="42" t="s">
-        <v>1504</v>
+        <v>1503</v>
       </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A175" s="18" t="s">
-        <v>1149</v>
+        <v>1148</v>
       </c>
       <c r="B175" s="18" t="s">
         <v>73</v>
@@ -7477,12 +7477,12 @@
         <v>422</v>
       </c>
       <c r="D175" s="42" t="s">
-        <v>1504</v>
+        <v>1503</v>
       </c>
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A176" s="18" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
       <c r="B176" s="18" t="s">
         <v>99</v>
@@ -7491,12 +7491,12 @@
         <v>422</v>
       </c>
       <c r="D176" s="42" t="s">
-        <v>1505</v>
+        <v>1504</v>
       </c>
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A177" s="18" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="B177" s="18" t="s">
         <v>74</v>
@@ -7505,12 +7505,12 @@
         <v>422</v>
       </c>
       <c r="D177" s="42" t="s">
-        <v>1505</v>
+        <v>1504</v>
       </c>
     </row>
     <row r="178" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A178" s="18" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
       <c r="B178" s="18" t="s">
         <v>86</v>
@@ -7519,12 +7519,12 @@
         <v>422</v>
       </c>
       <c r="D178" s="42" t="s">
-        <v>1505</v>
+        <v>1504</v>
       </c>
     </row>
     <row r="179" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A179" s="18" t="s">
-        <v>1153</v>
+        <v>1152</v>
       </c>
       <c r="B179" s="18" t="s">
         <v>100</v>
@@ -7533,12 +7533,12 @@
         <v>422</v>
       </c>
       <c r="D179" s="42" t="s">
-        <v>1506</v>
+        <v>1505</v>
       </c>
     </row>
     <row r="180" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A180" s="18" t="s">
-        <v>1154</v>
+        <v>1153</v>
       </c>
       <c r="B180" s="18" t="s">
         <v>70</v>
@@ -7547,12 +7547,12 @@
         <v>422</v>
       </c>
       <c r="D180" s="42" t="s">
-        <v>1506</v>
+        <v>1505</v>
       </c>
     </row>
     <row r="181" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A181" s="18" t="s">
-        <v>1155</v>
+        <v>1154</v>
       </c>
       <c r="B181" s="18" t="s">
         <v>78</v>
@@ -7561,12 +7561,12 @@
         <v>422</v>
       </c>
       <c r="D181" s="42" t="s">
-        <v>1506</v>
+        <v>1505</v>
       </c>
     </row>
     <row r="182" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A182" s="18" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
       <c r="B182" s="18" t="s">
         <v>90</v>
@@ -7575,12 +7575,12 @@
         <v>422</v>
       </c>
       <c r="D182" s="42" t="s">
-        <v>1507</v>
+        <v>1506</v>
       </c>
     </row>
     <row r="183" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A183" s="18" t="s">
-        <v>1157</v>
+        <v>1156</v>
       </c>
       <c r="B183" s="18" t="s">
         <v>104</v>
@@ -7589,12 +7589,12 @@
         <v>422</v>
       </c>
       <c r="D183" s="42" t="s">
-        <v>1507</v>
+        <v>1506</v>
       </c>
     </row>
     <row r="184" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A184" s="18" t="s">
-        <v>1158</v>
+        <v>1157</v>
       </c>
       <c r="B184" s="18" t="s">
         <v>112</v>
@@ -7603,12 +7603,12 @@
         <v>422</v>
       </c>
       <c r="D184" s="42" t="s">
-        <v>1508</v>
+        <v>1507</v>
       </c>
     </row>
     <row r="185" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A185" s="18" t="s">
-        <v>1159</v>
+        <v>1158</v>
       </c>
       <c r="B185" s="18" t="s">
         <v>80</v>
@@ -7617,12 +7617,12 @@
         <v>422</v>
       </c>
       <c r="D185" s="42" t="s">
-        <v>1508</v>
+        <v>1507</v>
       </c>
     </row>
     <row r="186" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A186" s="18" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="B186" s="18" t="s">
         <v>95</v>
@@ -7631,12 +7631,12 @@
         <v>422</v>
       </c>
       <c r="D186" s="42" t="s">
-        <v>1509</v>
+        <v>1508</v>
       </c>
     </row>
     <row r="187" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A187" s="18" t="s">
-        <v>1161</v>
+        <v>1160</v>
       </c>
       <c r="B187" s="18" t="s">
         <v>81</v>
@@ -7645,12 +7645,12 @@
         <v>422</v>
       </c>
       <c r="D187" s="42" t="s">
-        <v>1509</v>
+        <v>1508</v>
       </c>
     </row>
     <row r="188" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A188" s="18" t="s">
-        <v>1162</v>
+        <v>1161</v>
       </c>
       <c r="B188" s="18" t="s">
         <v>117</v>
@@ -7659,12 +7659,12 @@
         <v>422</v>
       </c>
       <c r="D188" s="42" t="s">
-        <v>1510</v>
+        <v>1509</v>
       </c>
     </row>
     <row r="189" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A189" s="18" t="s">
-        <v>1163</v>
+        <v>1162</v>
       </c>
       <c r="B189" s="18" t="s">
         <v>91</v>
@@ -7673,12 +7673,12 @@
         <v>422</v>
       </c>
       <c r="D189" s="42" t="s">
-        <v>1510</v>
+        <v>1509</v>
       </c>
     </row>
     <row r="190" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A190" s="18" t="s">
-        <v>1164</v>
+        <v>1163</v>
       </c>
       <c r="B190" s="18" t="s">
         <v>120</v>
@@ -7687,12 +7687,12 @@
         <v>422</v>
       </c>
       <c r="D190" s="42" t="s">
-        <v>1511</v>
+        <v>1510</v>
       </c>
     </row>
     <row r="191" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A191" s="18" t="s">
-        <v>1165</v>
+        <v>1164</v>
       </c>
       <c r="B191" s="18" t="s">
         <v>119</v>
@@ -7701,12 +7701,12 @@
         <v>422</v>
       </c>
       <c r="D191" s="42" t="s">
-        <v>1511</v>
+        <v>1510</v>
       </c>
     </row>
     <row r="192" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A192" s="18" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
       <c r="B192" s="18" t="s">
         <v>93</v>
@@ -7715,12 +7715,12 @@
         <v>422</v>
       </c>
       <c r="D192" s="42" t="s">
-        <v>1512</v>
+        <v>1511</v>
       </c>
     </row>
     <row r="193" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A193" s="18" t="s">
-        <v>1167</v>
+        <v>1166</v>
       </c>
       <c r="B193" s="18" t="s">
         <v>94</v>
@@ -7729,7 +7729,7 @@
         <v>422</v>
       </c>
       <c r="D193" s="42" t="s">
-        <v>1512</v>
+        <v>1511</v>
       </c>
     </row>
     <row r="194" spans="1:4" x14ac:dyDescent="0.2">
@@ -10807,487 +10807,487 @@
     </row>
     <row r="301" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A301" s="35" t="s">
-        <v>1168</v>
+        <v>1167</v>
       </c>
       <c r="F301" s="2"/>
     </row>
     <row r="302" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A302" s="35" t="s">
-        <v>1169</v>
+        <v>1168</v>
       </c>
       <c r="F302" s="2"/>
     </row>
     <row r="303" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A303" s="35" t="s">
-        <v>1170</v>
+        <v>1169</v>
       </c>
       <c r="F303" s="2"/>
     </row>
     <row r="304" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A304" s="35" t="s">
-        <v>1171</v>
+        <v>1170</v>
       </c>
       <c r="F304" s="2"/>
     </row>
     <row r="305" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A305" s="35" t="s">
-        <v>1172</v>
+        <v>1171</v>
       </c>
       <c r="F305" s="2"/>
     </row>
     <row r="306" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A306" s="35" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="F306" s="2"/>
     </row>
     <row r="307" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A307" s="35" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="F307" s="2"/>
     </row>
     <row r="308" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A308" s="35" t="s">
-        <v>1175</v>
+        <v>1174</v>
       </c>
       <c r="F308" s="2"/>
     </row>
     <row r="309" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A309" s="35" t="s">
-        <v>1176</v>
+        <v>1175</v>
       </c>
       <c r="F309" s="2"/>
     </row>
     <row r="310" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A310" s="35" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="F310" s="2"/>
     </row>
     <row r="311" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A311" s="35" t="s">
-        <v>1178</v>
+        <v>1177</v>
       </c>
       <c r="F311" s="2"/>
     </row>
     <row r="312" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A312" s="35" t="s">
-        <v>1179</v>
+        <v>1178</v>
       </c>
       <c r="F312" s="2"/>
     </row>
     <row r="313" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A313" s="35" t="s">
-        <v>1180</v>
+        <v>1179</v>
       </c>
       <c r="F313" s="2"/>
     </row>
     <row r="314" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A314" s="35" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
       <c r="F314" s="2"/>
     </row>
     <row r="315" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A315" s="35" t="s">
-        <v>1182</v>
+        <v>1181</v>
       </c>
       <c r="F315" s="2"/>
     </row>
     <row r="316" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A316" s="35" t="s">
-        <v>1183</v>
+        <v>1182</v>
       </c>
       <c r="F316" s="2"/>
     </row>
     <row r="317" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A317" s="35" t="s">
-        <v>1184</v>
+        <v>1183</v>
       </c>
       <c r="F317" s="2"/>
     </row>
     <row r="318" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A318" s="35" t="s">
-        <v>1185</v>
+        <v>1184</v>
       </c>
       <c r="F318" s="2"/>
     </row>
     <row r="319" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A319" s="35" t="s">
-        <v>1186</v>
+        <v>1185</v>
       </c>
       <c r="F319" s="2"/>
     </row>
     <row r="320" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A320" s="35" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
       <c r="F320" s="2"/>
     </row>
     <row r="321" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A321" s="35" t="s">
-        <v>1188</v>
+        <v>1187</v>
       </c>
       <c r="F321" s="2"/>
     </row>
     <row r="322" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A322" s="35" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="F322" s="2"/>
     </row>
     <row r="323" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A323" s="35" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
       <c r="F323" s="2"/>
     </row>
     <row r="324" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A324" s="35" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
       <c r="F324" s="2"/>
     </row>
     <row r="325" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A325" s="35" t="s">
-        <v>1192</v>
+        <v>1191</v>
       </c>
       <c r="F325" s="2"/>
     </row>
     <row r="326" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A326" s="35" t="s">
-        <v>1193</v>
+        <v>1192</v>
       </c>
       <c r="F326" s="2"/>
     </row>
     <row r="327" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A327" s="35" t="s">
-        <v>1194</v>
+        <v>1193</v>
       </c>
       <c r="F327" s="2"/>
     </row>
     <row r="328" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A328" s="35" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
       <c r="F328" s="2"/>
     </row>
     <row r="329" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A329" s="35" t="s">
-        <v>1196</v>
+        <v>1195</v>
       </c>
       <c r="F329" s="2"/>
     </row>
     <row r="330" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A330" s="35" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
       <c r="F330" s="2"/>
     </row>
     <row r="331" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A331" s="35" t="s">
-        <v>1198</v>
+        <v>1197</v>
       </c>
       <c r="F331" s="2"/>
     </row>
     <row r="332" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A332" s="35" t="s">
-        <v>1199</v>
+        <v>1198</v>
       </c>
       <c r="F332" s="2"/>
     </row>
     <row r="333" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A333" s="35" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="F333" s="2"/>
     </row>
     <row r="334" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A334" s="35" t="s">
-        <v>1201</v>
+        <v>1200</v>
       </c>
       <c r="F334" s="2"/>
     </row>
     <row r="335" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A335" s="35" t="s">
-        <v>1202</v>
+        <v>1201</v>
       </c>
       <c r="F335" s="2"/>
     </row>
     <row r="336" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A336" s="35" t="s">
-        <v>1203</v>
+        <v>1202</v>
       </c>
       <c r="F336" s="2"/>
     </row>
     <row r="337" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A337" s="35" t="s">
-        <v>1204</v>
+        <v>1203</v>
       </c>
       <c r="F337" s="2"/>
     </row>
     <row r="338" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A338" s="35" t="s">
-        <v>1205</v>
+        <v>1204</v>
       </c>
       <c r="F338" s="2"/>
     </row>
     <row r="339" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A339" s="35" t="s">
-        <v>1206</v>
+        <v>1205</v>
       </c>
       <c r="F339" s="2"/>
     </row>
     <row r="340" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A340" s="35" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
       <c r="F340" s="2"/>
     </row>
     <row r="341" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A341" s="35" t="s">
-        <v>1208</v>
+        <v>1207</v>
       </c>
       <c r="F341" s="2"/>
     </row>
     <row r="342" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A342" s="35" t="s">
-        <v>1209</v>
+        <v>1208</v>
       </c>
       <c r="F342" s="2"/>
     </row>
     <row r="343" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A343" s="35" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="F343" s="2"/>
     </row>
     <row r="344" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A344" s="35" t="s">
-        <v>1211</v>
+        <v>1210</v>
       </c>
       <c r="F344" s="2"/>
     </row>
     <row r="345" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A345" s="35" t="s">
-        <v>1212</v>
+        <v>1211</v>
       </c>
       <c r="F345" s="2"/>
     </row>
     <row r="346" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A346" s="35" t="s">
-        <v>1213</v>
+        <v>1212</v>
       </c>
       <c r="F346" s="2"/>
     </row>
     <row r="347" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A347" s="35" t="s">
-        <v>1214</v>
+        <v>1213</v>
       </c>
       <c r="F347" s="2"/>
     </row>
     <row r="348" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A348" s="35" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="F348" s="2"/>
     </row>
     <row r="349" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A349" s="35" t="s">
-        <v>1216</v>
+        <v>1215</v>
       </c>
       <c r="F349" s="2"/>
     </row>
     <row r="350" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A350" s="35" t="s">
-        <v>1217</v>
+        <v>1216</v>
       </c>
       <c r="F350" s="2"/>
     </row>
     <row r="351" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A351" s="35" t="s">
-        <v>1218</v>
+        <v>1217</v>
       </c>
       <c r="F351" s="2"/>
     </row>
     <row r="352" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A352" s="35" t="s">
-        <v>1219</v>
+        <v>1218</v>
       </c>
       <c r="F352" s="2"/>
     </row>
     <row r="353" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A353" s="35" t="s">
-        <v>1220</v>
+        <v>1219</v>
       </c>
       <c r="F353" s="2"/>
     </row>
     <row r="354" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A354" s="35" t="s">
-        <v>1221</v>
+        <v>1220</v>
       </c>
       <c r="F354" s="2"/>
     </row>
     <row r="355" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A355" s="35" t="s">
-        <v>1222</v>
+        <v>1221</v>
       </c>
       <c r="F355" s="2"/>
     </row>
     <row r="356" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A356" s="35" t="s">
-        <v>1223</v>
+        <v>1222</v>
       </c>
       <c r="F356" s="2"/>
     </row>
     <row r="357" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A357" s="35" t="s">
-        <v>1224</v>
+        <v>1223</v>
       </c>
       <c r="F357" s="2"/>
     </row>
     <row r="358" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A358" s="35" t="s">
-        <v>1225</v>
+        <v>1224</v>
       </c>
       <c r="F358" s="2"/>
     </row>
     <row r="359" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A359" s="35" t="s">
-        <v>1226</v>
+        <v>1225</v>
       </c>
       <c r="F359" s="2"/>
     </row>
     <row r="360" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A360" s="35" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
       <c r="F360" s="2"/>
     </row>
     <row r="361" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A361" s="35" t="s">
-        <v>1228</v>
+        <v>1227</v>
       </c>
       <c r="F361" s="2"/>
     </row>
     <row r="362" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A362" s="35" t="s">
-        <v>1229</v>
+        <v>1228</v>
       </c>
       <c r="F362" s="2"/>
     </row>
     <row r="363" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A363" s="35" t="s">
-        <v>1230</v>
+        <v>1229</v>
       </c>
       <c r="F363" s="2"/>
     </row>
     <row r="364" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A364" s="35" t="s">
-        <v>1231</v>
+        <v>1230</v>
       </c>
       <c r="F364" s="2"/>
     </row>
     <row r="365" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A365" s="35" t="s">
-        <v>1232</v>
+        <v>1231</v>
       </c>
       <c r="F365" s="2"/>
     </row>
     <row r="366" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A366" s="35" t="s">
-        <v>1233</v>
+        <v>1232</v>
       </c>
       <c r="F366" s="2"/>
     </row>
     <row r="367" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A367" s="35" t="s">
-        <v>1234</v>
+        <v>1233</v>
       </c>
       <c r="F367" s="2"/>
     </row>
     <row r="368" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A368" s="35" t="s">
-        <v>1235</v>
+        <v>1234</v>
       </c>
       <c r="F368" s="2"/>
     </row>
     <row r="369" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A369" s="35" t="s">
-        <v>1236</v>
+        <v>1235</v>
       </c>
       <c r="F369" s="2"/>
     </row>
     <row r="370" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A370" s="35" t="s">
-        <v>1237</v>
+        <v>1236</v>
       </c>
       <c r="F370" s="2"/>
     </row>
     <row r="371" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A371" s="35" t="s">
-        <v>1238</v>
+        <v>1237</v>
       </c>
       <c r="F371" s="2"/>
     </row>
     <row r="372" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A372" s="35" t="s">
-        <v>1239</v>
+        <v>1238</v>
       </c>
       <c r="F372" s="2"/>
     </row>
     <row r="373" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A373" s="35" t="s">
-        <v>1240</v>
+        <v>1239</v>
       </c>
       <c r="F373" s="2"/>
     </row>
     <row r="374" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A374" s="35" t="s">
-        <v>1241</v>
+        <v>1240</v>
       </c>
       <c r="F374" s="2"/>
     </row>
     <row r="375" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A375" s="35" t="s">
-        <v>1242</v>
+        <v>1241</v>
       </c>
       <c r="F375" s="2"/>
     </row>
     <row r="376" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A376" s="35" t="s">
-        <v>1243</v>
+        <v>1242</v>
       </c>
       <c r="F376" s="2"/>
     </row>
     <row r="377" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A377" s="35" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="F377" s="2"/>
     </row>
     <row r="378" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A378" s="35" t="s">
-        <v>1245</v>
+        <v>1244</v>
       </c>
       <c r="F378" s="2"/>
     </row>
     <row r="379" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A379" s="35" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="F379" s="2"/>
     </row>
     <row r="380" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A380" s="35" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="F380" s="2"/>
     </row>
     <row r="381" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A381" s="35" t="s">
-        <v>1248</v>
+        <v>1247</v>
       </c>
       <c r="F381" s="2"/>
     </row>
@@ -11299,73 +11299,73 @@
     </row>
     <row r="383" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A383" s="35" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="F383" s="2"/>
     </row>
     <row r="384" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A384" s="35" t="s">
-        <v>1250</v>
+        <v>1249</v>
       </c>
       <c r="F384" s="2"/>
     </row>
     <row r="385" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A385" s="35" t="s">
-        <v>1251</v>
+        <v>1250</v>
       </c>
       <c r="F385" s="2"/>
     </row>
     <row r="386" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A386" s="35" t="s">
-        <v>1252</v>
+        <v>1251</v>
       </c>
       <c r="F386" s="2"/>
     </row>
     <row r="387" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A387" s="35" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="F387" s="2"/>
     </row>
     <row r="388" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A388" s="35" t="s">
-        <v>1254</v>
+        <v>1253</v>
       </c>
       <c r="F388" s="2"/>
     </row>
     <row r="389" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A389" s="35" t="s">
-        <v>1255</v>
+        <v>1254</v>
       </c>
       <c r="F389" s="2"/>
     </row>
     <row r="390" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A390" s="35" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
       <c r="F390" s="2"/>
     </row>
     <row r="391" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A391" s="35" t="s">
-        <v>1257</v>
+        <v>1256</v>
       </c>
       <c r="F391" s="2"/>
     </row>
     <row r="392" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A392" s="35" t="s">
-        <v>1258</v>
+        <v>1257</v>
       </c>
       <c r="F392" s="2"/>
     </row>
     <row r="393" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A393" s="35" t="s">
-        <v>1259</v>
+        <v>1258</v>
       </c>
       <c r="F393" s="2"/>
     </row>
     <row r="394" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A394" s="35" t="s">
-        <v>1260</v>
+        <v>1259</v>
       </c>
       <c r="D394" s="20"/>
       <c r="E394" s="20"/>
@@ -11374,7 +11374,7 @@
     </row>
     <row r="395" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A395" s="35" t="s">
-        <v>1261</v>
+        <v>1260</v>
       </c>
       <c r="D395" s="20"/>
       <c r="E395" s="20"/>
@@ -11383,7 +11383,7 @@
     </row>
     <row r="396" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A396" s="35" t="s">
-        <v>1262</v>
+        <v>1261</v>
       </c>
       <c r="D396" s="20"/>
       <c r="E396" s="20"/>
@@ -11392,7 +11392,7 @@
     </row>
     <row r="397" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A397" s="35" t="s">
-        <v>1263</v>
+        <v>1262</v>
       </c>
       <c r="D397" s="20"/>
       <c r="E397" s="20"/>
@@ -11401,7 +11401,7 @@
     </row>
     <row r="398" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A398" s="35" t="s">
-        <v>1264</v>
+        <v>1263</v>
       </c>
       <c r="D398" s="20"/>
       <c r="E398" s="20"/>
@@ -11410,7 +11410,7 @@
     </row>
     <row r="399" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A399" s="35" t="s">
-        <v>1265</v>
+        <v>1264</v>
       </c>
       <c r="D399" s="20"/>
       <c r="E399" s="20"/>
@@ -11419,7 +11419,7 @@
     </row>
     <row r="400" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A400" s="35" t="s">
-        <v>1266</v>
+        <v>1265</v>
       </c>
       <c r="D400" s="20"/>
       <c r="E400" s="20"/>
@@ -11428,7 +11428,7 @@
     </row>
     <row r="401" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A401" s="35" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="D401" s="20"/>
       <c r="E401" s="20"/>
@@ -11437,7 +11437,7 @@
     </row>
     <row r="402" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A402" s="35" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
       <c r="D402" s="20"/>
       <c r="E402" s="20"/>
@@ -11446,7 +11446,7 @@
     </row>
     <row r="403" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A403" s="35" t="s">
-        <v>1269</v>
+        <v>1268</v>
       </c>
       <c r="D403" s="20"/>
       <c r="E403" s="20"/>
@@ -11455,7 +11455,7 @@
     </row>
     <row r="404" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A404" s="35" t="s">
-        <v>1270</v>
+        <v>1269</v>
       </c>
       <c r="D404" s="20"/>
       <c r="E404" s="20"/>
@@ -11464,7 +11464,7 @@
     </row>
     <row r="405" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A405" s="35" t="s">
-        <v>1271</v>
+        <v>1270</v>
       </c>
       <c r="D405" s="20"/>
       <c r="E405" s="20"/>
@@ -11473,7 +11473,7 @@
     </row>
     <row r="406" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A406" s="35" t="s">
-        <v>1272</v>
+        <v>1271</v>
       </c>
       <c r="D406" s="20"/>
       <c r="E406" s="20"/>
@@ -11482,7 +11482,7 @@
     </row>
     <row r="407" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A407" s="35" t="s">
-        <v>1273</v>
+        <v>1272</v>
       </c>
       <c r="D407" s="20"/>
       <c r="E407" s="20"/>
@@ -11491,7 +11491,7 @@
     </row>
     <row r="408" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A408" s="35" t="s">
-        <v>1274</v>
+        <v>1273</v>
       </c>
       <c r="D408" s="20"/>
       <c r="E408" s="20"/>
@@ -11500,7 +11500,7 @@
     </row>
     <row r="409" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A409" s="35" t="s">
-        <v>1275</v>
+        <v>1274</v>
       </c>
       <c r="D409" s="20"/>
       <c r="E409" s="20"/>
@@ -11509,7 +11509,7 @@
     </row>
     <row r="410" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A410" s="35" t="s">
-        <v>1276</v>
+        <v>1275</v>
       </c>
       <c r="D410" s="20"/>
       <c r="E410" s="20"/>
@@ -11518,7 +11518,7 @@
     </row>
     <row r="411" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A411" s="35" t="s">
-        <v>1277</v>
+        <v>1276</v>
       </c>
       <c r="D411" s="20"/>
       <c r="E411" s="20"/>
@@ -11527,7 +11527,7 @@
     </row>
     <row r="412" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A412" s="35" t="s">
-        <v>1278</v>
+        <v>1277</v>
       </c>
       <c r="D412" s="20"/>
       <c r="E412" s="20"/>
@@ -11536,7 +11536,7 @@
     </row>
     <row r="413" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A413" s="35" t="s">
-        <v>1279</v>
+        <v>1278</v>
       </c>
       <c r="D413" s="20"/>
       <c r="E413" s="20"/>
@@ -11545,7 +11545,7 @@
     </row>
     <row r="414" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A414" s="35" t="s">
-        <v>1280</v>
+        <v>1279</v>
       </c>
       <c r="D414" s="20"/>
       <c r="E414" s="20"/>
@@ -11554,7 +11554,7 @@
     </row>
     <row r="415" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A415" s="35" t="s">
-        <v>1281</v>
+        <v>1280</v>
       </c>
       <c r="D415" s="20"/>
       <c r="E415" s="20"/>
@@ -11563,7 +11563,7 @@
     </row>
     <row r="416" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A416" s="35" t="s">
-        <v>1282</v>
+        <v>1281</v>
       </c>
       <c r="D416" s="20"/>
       <c r="E416" s="20"/>
@@ -11572,7 +11572,7 @@
     </row>
     <row r="417" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A417" s="35" t="s">
-        <v>1283</v>
+        <v>1282</v>
       </c>
       <c r="D417" s="20"/>
       <c r="E417" s="20"/>
@@ -11581,7 +11581,7 @@
     </row>
     <row r="418" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A418" s="35" t="s">
-        <v>1284</v>
+        <v>1283</v>
       </c>
       <c r="D418" s="20"/>
       <c r="E418" s="20"/>
@@ -11590,7 +11590,7 @@
     </row>
     <row r="419" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A419" s="35" t="s">
-        <v>1285</v>
+        <v>1284</v>
       </c>
       <c r="D419" s="20"/>
       <c r="E419" s="20"/>
@@ -11599,7 +11599,7 @@
     </row>
     <row r="420" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A420" s="35" t="s">
-        <v>1286</v>
+        <v>1285</v>
       </c>
       <c r="D420" s="20"/>
       <c r="E420" s="20"/>
@@ -11608,7 +11608,7 @@
     </row>
     <row r="421" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A421" s="35" t="s">
-        <v>1287</v>
+        <v>1286</v>
       </c>
       <c r="D421" s="20"/>
       <c r="E421" s="20"/>
@@ -11617,7 +11617,7 @@
     </row>
     <row r="422" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A422" s="35" t="s">
-        <v>1288</v>
+        <v>1287</v>
       </c>
       <c r="D422" s="20"/>
       <c r="E422" s="20"/>
@@ -11626,7 +11626,7 @@
     </row>
     <row r="423" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A423" s="35" t="s">
-        <v>1289</v>
+        <v>1288</v>
       </c>
       <c r="D423" s="20"/>
       <c r="E423" s="20"/>
@@ -11635,7 +11635,7 @@
     </row>
     <row r="424" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A424" s="35" t="s">
-        <v>1290</v>
+        <v>1289</v>
       </c>
       <c r="D424" s="20"/>
       <c r="E424" s="20"/>
@@ -11644,7 +11644,7 @@
     </row>
     <row r="425" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A425" s="35" t="s">
-        <v>1291</v>
+        <v>1290</v>
       </c>
       <c r="D425" s="20"/>
       <c r="E425" s="20"/>
@@ -11653,7 +11653,7 @@
     </row>
     <row r="426" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A426" s="35" t="s">
-        <v>1292</v>
+        <v>1291</v>
       </c>
       <c r="D426" s="20"/>
       <c r="E426" s="20"/>
@@ -11662,7 +11662,7 @@
     </row>
     <row r="427" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A427" s="35" t="s">
-        <v>1293</v>
+        <v>1292</v>
       </c>
       <c r="D427" s="20"/>
       <c r="E427" s="20"/>
@@ -11671,7 +11671,7 @@
     </row>
     <row r="428" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A428" s="35" t="s">
-        <v>1294</v>
+        <v>1293</v>
       </c>
       <c r="D428" s="20"/>
       <c r="E428" s="20"/>
@@ -11680,7 +11680,7 @@
     </row>
     <row r="429" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A429" s="35" t="s">
-        <v>1295</v>
+        <v>1294</v>
       </c>
       <c r="D429" s="20"/>
       <c r="E429" s="20"/>
@@ -11689,7 +11689,7 @@
     </row>
     <row r="430" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A430" s="35" t="s">
-        <v>1296</v>
+        <v>1295</v>
       </c>
       <c r="D430" s="20"/>
       <c r="E430" s="20"/>
@@ -11698,7 +11698,7 @@
     </row>
     <row r="431" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A431" s="35" t="s">
-        <v>1297</v>
+        <v>1296</v>
       </c>
       <c r="D431" s="20"/>
       <c r="E431" s="20"/>
@@ -11716,7 +11716,7 @@
     </row>
     <row r="433" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A433" s="35" t="s">
-        <v>1298</v>
+        <v>1297</v>
       </c>
       <c r="D433" s="20"/>
       <c r="E433" s="20"/>
@@ -11725,7 +11725,7 @@
     </row>
     <row r="434" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A434" s="35" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
       <c r="D434" s="20"/>
       <c r="E434" s="20"/>
@@ -11734,7 +11734,7 @@
     </row>
     <row r="435" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A435" s="35" t="s">
-        <v>1300</v>
+        <v>1299</v>
       </c>
       <c r="D435" s="20"/>
       <c r="E435" s="20"/>
@@ -11743,7 +11743,7 @@
     </row>
     <row r="436" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A436" s="35" t="s">
-        <v>1301</v>
+        <v>1300</v>
       </c>
       <c r="D436" s="20"/>
       <c r="E436" s="20"/>
@@ -11752,7 +11752,7 @@
     </row>
     <row r="437" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A437" s="35" t="s">
-        <v>1302</v>
+        <v>1301</v>
       </c>
       <c r="D437" s="20"/>
       <c r="E437" s="20"/>
@@ -11761,7 +11761,7 @@
     </row>
     <row r="438" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A438" s="35" t="s">
-        <v>1303</v>
+        <v>1302</v>
       </c>
       <c r="D438" s="20"/>
       <c r="E438" s="20"/>
@@ -11770,7 +11770,7 @@
     </row>
     <row r="439" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A439" s="35" t="s">
-        <v>1304</v>
+        <v>1303</v>
       </c>
       <c r="D439" s="20"/>
       <c r="E439" s="20"/>
@@ -11779,7 +11779,7 @@
     </row>
     <row r="440" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A440" s="35" t="s">
-        <v>1305</v>
+        <v>1304</v>
       </c>
       <c r="D440" s="20"/>
       <c r="E440" s="20"/>
@@ -11788,7 +11788,7 @@
     </row>
     <row r="441" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A441" s="35" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="D441" s="20"/>
       <c r="E441" s="20"/>
@@ -11806,7 +11806,7 @@
     </row>
     <row r="443" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A443" s="35" t="s">
-        <v>1307</v>
+        <v>1306</v>
       </c>
       <c r="D443" s="20"/>
       <c r="E443" s="20"/>
@@ -11815,7 +11815,7 @@
     </row>
     <row r="444" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A444" s="35" t="s">
-        <v>1308</v>
+        <v>1307</v>
       </c>
       <c r="D444" s="20"/>
       <c r="E444" s="20"/>
@@ -11824,7 +11824,7 @@
     </row>
     <row r="445" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A445" s="35" t="s">
-        <v>1309</v>
+        <v>1308</v>
       </c>
       <c r="D445" s="20"/>
       <c r="E445" s="20"/>
@@ -11833,7 +11833,7 @@
     </row>
     <row r="446" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A446" s="35" t="s">
-        <v>1310</v>
+        <v>1309</v>
       </c>
       <c r="D446" s="20"/>
       <c r="E446" s="20"/>
@@ -11842,7 +11842,7 @@
     </row>
     <row r="447" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A447" s="35" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="D447" s="20"/>
       <c r="E447" s="20"/>
@@ -11851,7 +11851,7 @@
     </row>
     <row r="448" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A448" s="35" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
       <c r="D448" s="20"/>
       <c r="E448" s="20"/>
@@ -11860,7 +11860,7 @@
     </row>
     <row r="449" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A449" s="35" t="s">
-        <v>1313</v>
+        <v>1312</v>
       </c>
       <c r="D449" s="20"/>
       <c r="E449" s="20"/>
@@ -11869,7 +11869,7 @@
     </row>
     <row r="450" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A450" s="35" t="s">
-        <v>1314</v>
+        <v>1313</v>
       </c>
       <c r="D450" s="20"/>
       <c r="E450" s="20"/>
@@ -11878,7 +11878,7 @@
     </row>
     <row r="451" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A451" s="35" t="s">
-        <v>1315</v>
+        <v>1314</v>
       </c>
       <c r="D451" s="20"/>
       <c r="E451" s="20"/>
@@ -11887,7 +11887,7 @@
     </row>
     <row r="452" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A452" s="35" t="s">
-        <v>1316</v>
+        <v>1315</v>
       </c>
       <c r="D452" s="20"/>
       <c r="E452" s="20"/>
@@ -11896,7 +11896,7 @@
     </row>
     <row r="453" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A453" s="35" t="s">
-        <v>1317</v>
+        <v>1316</v>
       </c>
       <c r="D453" s="20"/>
       <c r="E453" s="20"/>
@@ -11905,7 +11905,7 @@
     </row>
     <row r="454" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A454" s="35" t="s">
-        <v>1318</v>
+        <v>1317</v>
       </c>
       <c r="D454" s="20"/>
       <c r="E454" s="20"/>
@@ -11914,7 +11914,7 @@
     </row>
     <row r="455" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A455" s="35" t="s">
-        <v>1319</v>
+        <v>1318</v>
       </c>
       <c r="D455" s="20"/>
       <c r="E455" s="20"/>
@@ -11923,7 +11923,7 @@
     </row>
     <row r="456" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A456" s="35" t="s">
-        <v>1320</v>
+        <v>1319</v>
       </c>
       <c r="D456" s="20"/>
       <c r="E456" s="20"/>
@@ -11932,7 +11932,7 @@
     </row>
     <row r="457" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A457" s="35" t="s">
-        <v>1321</v>
+        <v>1320</v>
       </c>
       <c r="D457" s="20"/>
       <c r="E457" s="20"/>
@@ -11941,7 +11941,7 @@
     </row>
     <row r="458" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A458" s="35" t="s">
-        <v>1322</v>
+        <v>1321</v>
       </c>
       <c r="D458" s="20"/>
       <c r="E458" s="20"/>
@@ -11950,7 +11950,7 @@
     </row>
     <row r="459" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A459" s="35" t="s">
-        <v>1323</v>
+        <v>1322</v>
       </c>
       <c r="D459" s="20"/>
       <c r="E459" s="20"/>
@@ -11959,7 +11959,7 @@
     </row>
     <row r="460" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A460" s="35" t="s">
-        <v>1324</v>
+        <v>1323</v>
       </c>
       <c r="D460" s="20"/>
       <c r="E460" s="20"/>
@@ -11968,7 +11968,7 @@
     </row>
     <row r="461" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A461" s="35" t="s">
-        <v>1325</v>
+        <v>1324</v>
       </c>
       <c r="D461" s="20"/>
       <c r="E461" s="20"/>
@@ -11977,7 +11977,7 @@
     </row>
     <row r="462" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A462" s="35" t="s">
-        <v>1326</v>
+        <v>1325</v>
       </c>
       <c r="D462" s="20"/>
       <c r="E462" s="20"/>
@@ -11986,7 +11986,7 @@
     </row>
     <row r="463" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A463" s="35" t="s">
-        <v>1327</v>
+        <v>1326</v>
       </c>
       <c r="D463" s="20"/>
       <c r="E463" s="20"/>
@@ -11995,7 +11995,7 @@
     </row>
     <row r="464" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A464" s="35" t="s">
-        <v>1328</v>
+        <v>1327</v>
       </c>
       <c r="D464" s="20"/>
       <c r="E464" s="20"/>
@@ -12004,7 +12004,7 @@
     </row>
     <row r="465" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A465" s="35" t="s">
-        <v>1329</v>
+        <v>1328</v>
       </c>
       <c r="D465" s="20"/>
       <c r="E465" s="20"/>
@@ -12013,7 +12013,7 @@
     </row>
     <row r="466" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A466" s="35" t="s">
-        <v>1330</v>
+        <v>1329</v>
       </c>
       <c r="D466" s="20"/>
       <c r="E466" s="20"/>
@@ -12022,7 +12022,7 @@
     </row>
     <row r="467" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A467" s="35" t="s">
-        <v>1331</v>
+        <v>1330</v>
       </c>
       <c r="D467" s="20"/>
       <c r="E467" s="20"/>
@@ -12031,7 +12031,7 @@
     </row>
     <row r="468" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A468" s="35" t="s">
-        <v>1332</v>
+        <v>1331</v>
       </c>
       <c r="D468" s="20"/>
       <c r="E468" s="20"/>
@@ -12040,7 +12040,7 @@
     </row>
     <row r="469" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A469" s="35" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="D469" s="20"/>
       <c r="E469" s="20"/>
@@ -12049,7 +12049,7 @@
     </row>
     <row r="470" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A470" s="35" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
       <c r="D470" s="20"/>
       <c r="E470" s="20"/>
@@ -12058,139 +12058,139 @@
     </row>
     <row r="471" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A471" s="35" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="F471" s="2"/>
     </row>
     <row r="472" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A472" s="35" t="s">
-        <v>1336</v>
+        <v>1335</v>
       </c>
       <c r="F472" s="2"/>
     </row>
     <row r="473" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A473" s="35" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="F473" s="2"/>
     </row>
     <row r="474" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A474" s="35" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="F474" s="2"/>
     </row>
     <row r="475" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A475" s="35" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
       <c r="F475" s="2"/>
     </row>
     <row r="476" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A476" s="35" t="s">
-        <v>1340</v>
+        <v>1339</v>
       </c>
       <c r="F476" s="2"/>
     </row>
     <row r="477" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A477" s="35" t="s">
-        <v>1341</v>
+        <v>1340</v>
       </c>
       <c r="F477" s="2"/>
     </row>
     <row r="478" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A478" s="35" t="s">
-        <v>1342</v>
+        <v>1341</v>
       </c>
       <c r="F478" s="2"/>
     </row>
     <row r="479" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A479" s="35" t="s">
-        <v>1343</v>
+        <v>1342</v>
       </c>
       <c r="F479" s="2"/>
     </row>
     <row r="480" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A480" s="35" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="F480" s="2"/>
     </row>
     <row r="481" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A481" s="35" t="s">
-        <v>1345</v>
+        <v>1344</v>
       </c>
       <c r="F481" s="2"/>
     </row>
     <row r="482" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A482" s="35" t="s">
-        <v>1346</v>
+        <v>1345</v>
       </c>
       <c r="F482" s="2"/>
     </row>
     <row r="483" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A483" s="35" t="s">
-        <v>1347</v>
+        <v>1346</v>
       </c>
       <c r="F483" s="2"/>
     </row>
     <row r="484" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A484" s="35" t="s">
-        <v>1348</v>
+        <v>1347</v>
       </c>
       <c r="F484" s="2"/>
     </row>
     <row r="485" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A485" s="35" t="s">
-        <v>1349</v>
+        <v>1348</v>
       </c>
       <c r="F485" s="2"/>
     </row>
     <row r="486" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A486" s="35" t="s">
-        <v>1350</v>
+        <v>1349</v>
       </c>
       <c r="F486" s="2"/>
     </row>
     <row r="487" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A487" s="35" t="s">
-        <v>1351</v>
+        <v>1350</v>
       </c>
       <c r="F487" s="2"/>
     </row>
     <row r="488" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A488" s="35" t="s">
-        <v>1352</v>
+        <v>1351</v>
       </c>
       <c r="F488" s="2"/>
     </row>
     <row r="489" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A489" s="35" t="s">
-        <v>1353</v>
+        <v>1352</v>
       </c>
       <c r="F489" s="2"/>
     </row>
     <row r="490" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A490" s="35" t="s">
-        <v>1354</v>
+        <v>1353</v>
       </c>
       <c r="F490" s="2"/>
     </row>
     <row r="491" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A491" s="35" t="s">
-        <v>1355</v>
+        <v>1354</v>
       </c>
       <c r="F491" s="2"/>
     </row>
     <row r="492" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A492" s="35" t="s">
-        <v>1356</v>
+        <v>1355</v>
       </c>
       <c r="F492" s="2"/>
     </row>
     <row r="493" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A493" s="35" t="s">
-        <v>1357</v>
+        <v>1356</v>
       </c>
       <c r="F493" s="2"/>
     </row>
@@ -12202,31 +12202,31 @@
     </row>
     <row r="495" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A495" s="35" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="F495" s="2"/>
     </row>
     <row r="496" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A496" s="35" t="s">
-        <v>1359</v>
+        <v>1358</v>
       </c>
       <c r="F496" s="2"/>
     </row>
     <row r="497" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A497" s="35" t="s">
-        <v>1360</v>
+        <v>1359</v>
       </c>
       <c r="F497" s="2"/>
     </row>
     <row r="498" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A498" s="35" t="s">
-        <v>1361</v>
+        <v>1360</v>
       </c>
       <c r="F498" s="2"/>
     </row>
     <row r="499" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A499" s="35" t="s">
-        <v>1362</v>
+        <v>1361</v>
       </c>
       <c r="F499" s="2"/>
     </row>
@@ -12238,127 +12238,127 @@
     </row>
     <row r="501" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A501" s="35" t="s">
-        <v>1363</v>
+        <v>1362</v>
       </c>
       <c r="F501" s="2"/>
     </row>
     <row r="502" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A502" s="35" t="s">
-        <v>1364</v>
+        <v>1363</v>
       </c>
       <c r="F502" s="2"/>
     </row>
     <row r="503" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A503" s="35" t="s">
-        <v>1365</v>
+        <v>1364</v>
       </c>
       <c r="F503" s="2"/>
     </row>
     <row r="504" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A504" s="35" t="s">
-        <v>1366</v>
+        <v>1365</v>
       </c>
       <c r="F504" s="2"/>
     </row>
     <row r="505" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A505" s="35" t="s">
-        <v>1367</v>
+        <v>1366</v>
       </c>
       <c r="F505" s="2"/>
     </row>
     <row r="506" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A506" s="35" t="s">
-        <v>1368</v>
+        <v>1367</v>
       </c>
       <c r="F506" s="2"/>
     </row>
     <row r="507" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A507" s="35" t="s">
-        <v>1369</v>
+        <v>1368</v>
       </c>
       <c r="F507" s="2"/>
     </row>
     <row r="508" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A508" s="35" t="s">
-        <v>1370</v>
+        <v>1369</v>
       </c>
       <c r="F508" s="2"/>
     </row>
     <row r="509" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A509" s="35" t="s">
-        <v>1371</v>
+        <v>1370</v>
       </c>
       <c r="F509" s="2"/>
     </row>
     <row r="510" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A510" s="35" t="s">
-        <v>1372</v>
+        <v>1371</v>
       </c>
       <c r="F510" s="2"/>
     </row>
     <row r="511" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A511" s="35" t="s">
-        <v>1373</v>
+        <v>1372</v>
       </c>
       <c r="F511" s="2"/>
     </row>
     <row r="512" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A512" s="35" t="s">
-        <v>1374</v>
+        <v>1373</v>
       </c>
       <c r="F512" s="2"/>
     </row>
     <row r="513" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A513" s="35" t="s">
-        <v>1375</v>
+        <v>1374</v>
       </c>
       <c r="F513" s="2"/>
     </row>
     <row r="514" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A514" s="35" t="s">
-        <v>1376</v>
+        <v>1375</v>
       </c>
       <c r="F514" s="2"/>
     </row>
     <row r="515" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A515" s="35" t="s">
-        <v>1377</v>
+        <v>1376</v>
       </c>
       <c r="F515" s="2"/>
     </row>
     <row r="516" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A516" s="35" t="s">
-        <v>1378</v>
+        <v>1377</v>
       </c>
       <c r="F516" s="2"/>
     </row>
     <row r="517" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A517" s="35" t="s">
-        <v>1379</v>
+        <v>1378</v>
       </c>
       <c r="F517" s="2"/>
     </row>
     <row r="518" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A518" s="35" t="s">
-        <v>1380</v>
+        <v>1379</v>
       </c>
       <c r="F518" s="2"/>
     </row>
     <row r="519" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A519" s="35" t="s">
-        <v>1381</v>
+        <v>1380</v>
       </c>
       <c r="F519" s="2"/>
     </row>
     <row r="520" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A520" s="35" t="s">
-        <v>1382</v>
+        <v>1381</v>
       </c>
       <c r="F520" s="2"/>
     </row>
     <row r="521" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A521" s="35" t="s">
-        <v>1383</v>
+        <v>1382</v>
       </c>
       <c r="F521" s="2"/>
     </row>
@@ -12376,31 +12376,31 @@
     </row>
     <row r="524" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A524" s="35" t="s">
-        <v>1384</v>
+        <v>1383</v>
       </c>
       <c r="F524" s="2"/>
     </row>
     <row r="525" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A525" s="35" t="s">
-        <v>1385</v>
+        <v>1384</v>
       </c>
       <c r="F525" s="2"/>
     </row>
     <row r="526" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A526" s="35" t="s">
-        <v>1386</v>
+        <v>1385</v>
       </c>
       <c r="F526" s="2"/>
     </row>
     <row r="527" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A527" s="35" t="s">
-        <v>1387</v>
+        <v>1386</v>
       </c>
       <c r="F527" s="2"/>
     </row>
     <row r="528" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A528" s="35" t="s">
-        <v>1388</v>
+        <v>1387</v>
       </c>
       <c r="F528" s="2"/>
     </row>
@@ -12412,43 +12412,43 @@
     </row>
     <row r="530" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A530" s="35" t="s">
-        <v>1389</v>
+        <v>1388</v>
       </c>
       <c r="F530" s="2"/>
     </row>
     <row r="531" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A531" s="35" t="s">
-        <v>1390</v>
+        <v>1389</v>
       </c>
       <c r="F531" s="2"/>
     </row>
     <row r="532" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A532" s="35" t="s">
-        <v>1391</v>
+        <v>1390</v>
       </c>
       <c r="F532" s="2"/>
     </row>
     <row r="533" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A533" s="35" t="s">
-        <v>1392</v>
+        <v>1391</v>
       </c>
       <c r="F533" s="2"/>
     </row>
     <row r="534" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A534" s="35" t="s">
-        <v>1393</v>
+        <v>1392</v>
       </c>
       <c r="F534" s="2"/>
     </row>
     <row r="535" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A535" s="35" t="s">
-        <v>1394</v>
+        <v>1393</v>
       </c>
       <c r="F535" s="2"/>
     </row>
     <row r="536" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A536" s="35" t="s">
-        <v>1395</v>
+        <v>1394</v>
       </c>
       <c r="F536" s="2"/>
     </row>
@@ -12460,199 +12460,199 @@
     </row>
     <row r="538" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A538" s="35" t="s">
-        <v>1396</v>
+        <v>1395</v>
       </c>
       <c r="F538" s="2"/>
     </row>
     <row r="539" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A539" s="35" t="s">
-        <v>1397</v>
+        <v>1396</v>
       </c>
       <c r="F539" s="2"/>
     </row>
     <row r="540" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A540" s="35" t="s">
-        <v>1398</v>
+        <v>1397</v>
       </c>
       <c r="F540" s="2"/>
     </row>
     <row r="541" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A541" s="35" t="s">
-        <v>1399</v>
+        <v>1398</v>
       </c>
       <c r="F541" s="2"/>
     </row>
     <row r="542" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A542" s="35" t="s">
-        <v>1400</v>
+        <v>1399</v>
       </c>
       <c r="F542" s="2"/>
     </row>
     <row r="543" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A543" s="35" t="s">
-        <v>1401</v>
+        <v>1400</v>
       </c>
       <c r="F543" s="2"/>
     </row>
     <row r="544" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A544" s="35" t="s">
-        <v>1402</v>
+        <v>1401</v>
       </c>
       <c r="F544" s="2"/>
     </row>
     <row r="545" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A545" s="35" t="s">
-        <v>1403</v>
+        <v>1402</v>
       </c>
       <c r="F545" s="2"/>
     </row>
     <row r="546" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A546" s="35" t="s">
-        <v>1404</v>
+        <v>1403</v>
       </c>
       <c r="F546" s="2"/>
     </row>
     <row r="547" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A547" s="35" t="s">
-        <v>1405</v>
+        <v>1404</v>
       </c>
       <c r="F547" s="2"/>
     </row>
     <row r="548" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A548" s="35" t="s">
-        <v>1406</v>
+        <v>1405</v>
       </c>
       <c r="F548" s="2"/>
     </row>
     <row r="549" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A549" s="35" t="s">
-        <v>1407</v>
+        <v>1406</v>
       </c>
       <c r="F549" s="2"/>
     </row>
     <row r="550" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A550" s="35" t="s">
-        <v>1408</v>
+        <v>1407</v>
       </c>
       <c r="F550" s="2"/>
     </row>
     <row r="551" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A551" s="35" t="s">
-        <v>1409</v>
+        <v>1408</v>
       </c>
       <c r="F551" s="2"/>
     </row>
     <row r="552" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A552" s="35" t="s">
-        <v>1410</v>
+        <v>1409</v>
       </c>
       <c r="F552" s="2"/>
     </row>
     <row r="553" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A553" s="35" t="s">
-        <v>1411</v>
+        <v>1410</v>
       </c>
       <c r="F553" s="2"/>
     </row>
     <row r="554" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A554" s="35" t="s">
-        <v>1412</v>
+        <v>1411</v>
       </c>
       <c r="F554" s="2"/>
     </row>
     <row r="555" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A555" s="35" t="s">
-        <v>1413</v>
+        <v>1412</v>
       </c>
       <c r="F555" s="2"/>
     </row>
     <row r="556" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A556" s="35" t="s">
-        <v>1414</v>
+        <v>1413</v>
       </c>
       <c r="F556" s="2"/>
     </row>
     <row r="557" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A557" s="35" t="s">
-        <v>1415</v>
+        <v>1414</v>
       </c>
       <c r="F557" s="2"/>
     </row>
     <row r="558" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A558" s="35" t="s">
-        <v>1416</v>
+        <v>1415</v>
       </c>
       <c r="F558" s="2"/>
     </row>
     <row r="559" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A559" s="35" t="s">
-        <v>1417</v>
+        <v>1416</v>
       </c>
       <c r="F559" s="2"/>
     </row>
     <row r="560" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A560" s="35" t="s">
-        <v>1418</v>
+        <v>1417</v>
       </c>
       <c r="F560" s="2"/>
     </row>
     <row r="561" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A561" s="35" t="s">
-        <v>1419</v>
+        <v>1418</v>
       </c>
       <c r="F561" s="2"/>
     </row>
     <row r="562" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A562" s="35" t="s">
-        <v>1420</v>
+        <v>1419</v>
       </c>
       <c r="F562" s="2"/>
     </row>
     <row r="563" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A563" s="35" t="s">
-        <v>1421</v>
+        <v>1420</v>
       </c>
       <c r="F563" s="2"/>
     </row>
     <row r="564" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A564" s="35" t="s">
-        <v>1422</v>
+        <v>1421</v>
       </c>
       <c r="F564" s="2"/>
     </row>
     <row r="565" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A565" s="35" t="s">
-        <v>1423</v>
+        <v>1422</v>
       </c>
       <c r="F565" s="2"/>
     </row>
     <row r="566" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A566" s="35" t="s">
-        <v>1424</v>
+        <v>1423</v>
       </c>
       <c r="F566" s="2"/>
     </row>
     <row r="567" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A567" s="35" t="s">
-        <v>1425</v>
+        <v>1424</v>
       </c>
       <c r="F567" s="2"/>
     </row>
     <row r="568" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A568" s="35" t="s">
-        <v>1426</v>
+        <v>1425</v>
       </c>
       <c r="F568" s="2"/>
     </row>
     <row r="569" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A569" s="35" t="s">
-        <v>1427</v>
+        <v>1426</v>
       </c>
       <c r="F569" s="2"/>
     </row>
     <row r="570" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A570" s="35" t="s">
-        <v>1428</v>
+        <v>1427</v>
       </c>
       <c r="F570" s="2"/>
     </row>
@@ -12664,7 +12664,7 @@
     </row>
     <row r="572" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A572" s="35" t="s">
-        <v>1429</v>
+        <v>1428</v>
       </c>
       <c r="F572" s="2"/>
     </row>
@@ -12676,43 +12676,43 @@
     </row>
     <row r="574" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A574" s="35" t="s">
-        <v>1430</v>
+        <v>1429</v>
       </c>
       <c r="F574" s="2"/>
     </row>
     <row r="575" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A575" s="35" t="s">
-        <v>1431</v>
+        <v>1430</v>
       </c>
       <c r="F575" s="2"/>
     </row>
     <row r="576" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A576" s="35" t="s">
-        <v>1432</v>
+        <v>1431</v>
       </c>
       <c r="F576" s="2"/>
     </row>
     <row r="577" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A577" s="35" t="s">
-        <v>1433</v>
+        <v>1432</v>
       </c>
       <c r="F577" s="2"/>
     </row>
     <row r="578" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A578" s="35" t="s">
-        <v>1434</v>
+        <v>1433</v>
       </c>
       <c r="F578" s="2"/>
     </row>
     <row r="579" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A579" s="35" t="s">
-        <v>1435</v>
+        <v>1434</v>
       </c>
       <c r="F579" s="2"/>
     </row>
     <row r="580" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A580" s="35" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="F580" s="2"/>
     </row>
@@ -12724,103 +12724,103 @@
     </row>
     <row r="582" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A582" s="35" t="s">
-        <v>1437</v>
+        <v>1436</v>
       </c>
       <c r="F582" s="2"/>
     </row>
     <row r="583" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A583" s="35" t="s">
-        <v>1438</v>
+        <v>1437</v>
       </c>
       <c r="F583" s="2"/>
     </row>
     <row r="584" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A584" s="35" t="s">
-        <v>1439</v>
+        <v>1438</v>
       </c>
       <c r="F584" s="2"/>
     </row>
     <row r="585" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A585" s="35" t="s">
-        <v>1440</v>
+        <v>1439</v>
       </c>
       <c r="F585" s="2"/>
     </row>
     <row r="586" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A586" s="35" t="s">
-        <v>1441</v>
+        <v>1440</v>
       </c>
       <c r="F586" s="2"/>
     </row>
     <row r="587" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A587" s="35" t="s">
-        <v>1442</v>
+        <v>1441</v>
       </c>
       <c r="F587" s="2"/>
     </row>
     <row r="588" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A588" s="35" t="s">
-        <v>1443</v>
+        <v>1442</v>
       </c>
       <c r="F588" s="2"/>
     </row>
     <row r="589" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A589" s="35" t="s">
-        <v>1444</v>
+        <v>1443</v>
       </c>
       <c r="F589" s="2"/>
     </row>
     <row r="590" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A590" s="35" t="s">
-        <v>1445</v>
+        <v>1444</v>
       </c>
       <c r="F590" s="2"/>
     </row>
     <row r="591" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A591" s="35" t="s">
-        <v>1446</v>
+        <v>1445</v>
       </c>
       <c r="F591" s="2"/>
     </row>
     <row r="592" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A592" s="35" t="s">
-        <v>1447</v>
+        <v>1446</v>
       </c>
       <c r="F592" s="2"/>
     </row>
     <row r="593" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A593" s="35" t="s">
-        <v>1448</v>
+        <v>1447</v>
       </c>
       <c r="F593" s="2"/>
     </row>
     <row r="594" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A594" s="35" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="F594" s="2"/>
     </row>
     <row r="595" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A595" s="35" t="s">
-        <v>1450</v>
+        <v>1449</v>
       </c>
       <c r="F595" s="2"/>
     </row>
     <row r="596" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A596" s="35" t="s">
-        <v>1451</v>
+        <v>1450</v>
       </c>
       <c r="F596" s="2"/>
     </row>
     <row r="597" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A597" s="35" t="s">
-        <v>1452</v>
+        <v>1451</v>
       </c>
       <c r="F597" s="2"/>
     </row>
     <row r="598" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A598" s="35" t="s">
-        <v>1453</v>
+        <v>1452</v>
       </c>
       <c r="D598" s="20"/>
       <c r="E598" s="20"/>
@@ -12829,7 +12829,7 @@
     </row>
     <row r="599" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A599" s="35" t="s">
-        <v>1454</v>
+        <v>1453</v>
       </c>
       <c r="D599" s="20"/>
       <c r="E599" s="20"/>
@@ -12838,7 +12838,7 @@
     </row>
     <row r="600" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A600" s="35" t="s">
-        <v>1455</v>
+        <v>1454</v>
       </c>
       <c r="D600" s="20"/>
       <c r="E600" s="20"/>
@@ -12847,7 +12847,7 @@
     </row>
     <row r="601" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A601" s="35" t="s">
-        <v>1456</v>
+        <v>1455</v>
       </c>
       <c r="D601" s="20"/>
       <c r="E601" s="20"/>
@@ -12856,7 +12856,7 @@
     </row>
     <row r="602" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A602" s="35" t="s">
-        <v>1457</v>
+        <v>1456</v>
       </c>
       <c r="D602" s="20"/>
       <c r="E602" s="20"/>
@@ -12865,7 +12865,7 @@
     </row>
     <row r="603" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A603" s="35" t="s">
-        <v>1458</v>
+        <v>1457</v>
       </c>
       <c r="D603" s="20"/>
       <c r="E603" s="20"/>
@@ -12883,7 +12883,7 @@
     </row>
     <row r="605" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A605" s="35" t="s">
-        <v>1459</v>
+        <v>1458</v>
       </c>
       <c r="D605" s="20"/>
       <c r="E605" s="20"/>
@@ -12892,7 +12892,7 @@
     </row>
     <row r="606" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A606" s="35" t="s">
-        <v>1460</v>
+        <v>1459</v>
       </c>
       <c r="D606" s="20"/>
       <c r="E606" s="20"/>
@@ -12901,7 +12901,7 @@
     </row>
     <row r="607" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A607" s="35" t="s">
-        <v>1461</v>
+        <v>1460</v>
       </c>
       <c r="D607" s="20"/>
       <c r="E607" s="20"/>
@@ -12910,7 +12910,7 @@
     </row>
     <row r="608" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A608" s="35" t="s">
-        <v>1462</v>
+        <v>1461</v>
       </c>
       <c r="D608" s="20"/>
       <c r="E608" s="20"/>
@@ -12919,7 +12919,7 @@
     </row>
     <row r="609" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A609" s="35" t="s">
-        <v>1463</v>
+        <v>1462</v>
       </c>
       <c r="D609" s="20"/>
       <c r="E609" s="20"/>
@@ -12928,7 +12928,7 @@
     </row>
     <row r="610" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A610" s="35" t="s">
-        <v>1464</v>
+        <v>1463</v>
       </c>
       <c r="D610" s="20"/>
       <c r="E610" s="20"/>
@@ -12937,7 +12937,7 @@
     </row>
     <row r="611" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A611" s="35" t="s">
-        <v>1465</v>
+        <v>1464</v>
       </c>
       <c r="D611" s="20"/>
       <c r="E611" s="20"/>
@@ -12946,7 +12946,7 @@
     </row>
     <row r="612" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A612" s="35" t="s">
-        <v>1466</v>
+        <v>1465</v>
       </c>
       <c r="D612" s="20"/>
       <c r="E612" s="20"/>
@@ -12955,7 +12955,7 @@
     </row>
     <row r="613" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A613" s="35" t="s">
-        <v>1467</v>
+        <v>1466</v>
       </c>
     </row>
   </sheetData>

</xml_diff>